<commit_message>
fixed export data pdf, excel csv
</commit_message>
<xml_diff>
--- a/income_statement.xlsx
+++ b/income_statement.xlsx
@@ -421,7 +421,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -439,7 +439,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-05</t>
         </is>
       </c>
     </row>
@@ -459,7 +459,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1000</v>
+        <v>207482</v>
       </c>
     </row>
     <row r="6"/>
@@ -489,7 +489,7 @@
         </is>
       </c>
       <c r="B10" s="1" t="n">
-        <v>1000</v>
+        <v>207482</v>
       </c>
     </row>
     <row r="11"/>

</xml_diff>